<commit_message>
feat: remove outdated log files and enhance extraction pipeline
- Deleted multiple log files (log1.txt, log2.txt, log3.txt, log4.txt, log5.txt, log6.txt, logRETRY.txt, logWEBSCRAPER.txt) to streamline the logging process.
- Updated the extraction pipeline to ensure no references to the removed log files remain, improving overall efficiency.
- Enhanced the README with clearer instructions for running the extraction process, including logging and power management.
- Adjusted the extraction scripts to reflect the removal of unnecessary logging, focusing on essential output and error handling.
</commit_message>
<xml_diff>
--- a/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
+++ b/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
@@ -597,7 +597,7 @@
         <v>39</v>
       </c>
       <c r="E4" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         <v>18</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         <v>32</v>
       </c>
       <c r="E12" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1070,13 +1070,9 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>0</v>
       </c>
@@ -1113,7 +1109,7 @@
         <v>37</v>
       </c>
       <c r="E16" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1285,7 +1281,7 @@
         <v>9</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1973,7 +1969,7 @@
         <v>17</v>
       </c>
       <c r="E36" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -2059,7 +2055,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -2661,7 +2657,7 @@
         <v>13</v>
       </c>
       <c r="E52" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2790,7 +2786,7 @@
         <v>26</v>
       </c>
       <c r="E55" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2833,7 +2829,7 @@
         <v>12</v>
       </c>
       <c r="E56" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -3005,7 +3001,7 @@
         <v>8</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -3091,13 +3087,9 @@
         <v>11</v>
       </c>
       <c r="E62" t="n">
-        <v>11</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="n">
         <v>0</v>
       </c>
@@ -3349,7 +3341,7 @@
         <v>21</v>
       </c>
       <c r="E68" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -3392,7 +3384,7 @@
         <v>18</v>
       </c>
       <c r="E69" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -3435,7 +3427,7 @@
         <v>2</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3478,7 +3470,7 @@
         <v>11</v>
       </c>
       <c r="E71" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -3521,7 +3513,7 @@
         <v>15</v>
       </c>
       <c r="E72" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -3994,7 +3986,7 @@
         <v>14</v>
       </c>
       <c r="E83" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -4037,7 +4029,7 @@
         <v>13</v>
       </c>
       <c r="E84" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -4123,7 +4115,7 @@
         <v>21</v>
       </c>
       <c r="E86" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -4166,13 +4158,9 @@
         <v>20</v>
       </c>
       <c r="E87" t="n">
-        <v>20</v>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="n">
         <v>0</v>
       </c>
@@ -4252,13 +4240,9 @@
         <v>14</v>
       </c>
       <c r="E89" t="n">
-        <v>14</v>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
         <v>0</v>
       </c>
@@ -4596,7 +4580,7 @@
         <v>17</v>
       </c>
       <c r="E97" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -4854,7 +4838,7 @@
         <v>2</v>
       </c>
       <c r="E103" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -4897,13 +4881,9 @@
         <v>17</v>
       </c>
       <c r="E104" t="n">
-        <v>17</v>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="n">
         <v>0</v>
       </c>
@@ -4940,7 +4920,7 @@
         <v>14</v>
       </c>
       <c r="E105" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -5069,7 +5049,7 @@
         <v>2</v>
       </c>
       <c r="E108" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -5112,7 +5092,7 @@
         <v>18</v>
       </c>
       <c r="E109" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: enhance extraction pipeline and update performance metrics
- Removed outdated log files (p2_log1.txt, p2_log2.txt, p2_log3.txt, p2_log4.txt) to streamline the logging process.
- Updated the extraction pipeline to improve efficiency and added adaptive retry strategies for error handling.
- Enhanced performance metrics, processing a total of 1571 files with a 100% success rate.
- Adjusted extraction quality report to reflect the latest data, including average content length and files needing re-extraction.
- Improved error handling and logging for better tracking of extraction processes and API interactions.
</commit_message>
<xml_diff>
--- a/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
+++ b/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
@@ -642,11 +642,7 @@
       <c r="E5" t="n">
         <v>14</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>0</v>
       </c>
@@ -1029,11 +1025,7 @@
       <c r="E14" t="n">
         <v>18</v>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>0</v>
       </c>
@@ -1070,9 +1062,13 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
@@ -1455,11 +1451,7 @@
       <c r="E24" t="n">
         <v>36</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
         <v>0</v>
       </c>
@@ -1541,11 +1533,7 @@
       <c r="E26" t="n">
         <v>10</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
         <v>0</v>
       </c>
@@ -1627,11 +1615,7 @@
       <c r="E28" t="n">
         <v>26</v>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
         <v>0</v>
       </c>
@@ -1670,11 +1654,7 @@
       <c r="E29" t="n">
         <v>13</v>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>0</v>
       </c>
@@ -1928,11 +1908,7 @@
       <c r="E35" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
         <v>0</v>
       </c>
@@ -2014,11 +1990,7 @@
       <c r="E37" t="n">
         <v>4</v>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
         <v>0</v>
       </c>
@@ -2143,11 +2115,7 @@
       <c r="E40" t="n">
         <v>20</v>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
         <v>0</v>
       </c>
@@ -2229,11 +2197,7 @@
       <c r="E42" t="n">
         <v>30</v>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
         <v>0</v>
       </c>
@@ -2272,11 +2236,7 @@
       <c r="E43" t="n">
         <v>28</v>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>0</v>
       </c>
@@ -2401,11 +2361,7 @@
       <c r="E46" t="n">
         <v>12</v>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
         <v>0</v>
       </c>
@@ -2444,11 +2400,7 @@
       <c r="E47" t="n">
         <v>24</v>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
         <v>0</v>
       </c>
@@ -3087,9 +3039,13 @@
         <v>11</v>
       </c>
       <c r="E62" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" t="inlineStr"/>
+        <v>11</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
@@ -3128,11 +3084,7 @@
       <c r="E63" t="n">
         <v>1</v>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="n">
         <v>0</v>
       </c>
@@ -3171,11 +3123,7 @@
       <c r="E64" t="n">
         <v>17</v>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="n">
         <v>0</v>
       </c>
@@ -3255,13 +3203,9 @@
         <v>17</v>
       </c>
       <c r="E66" t="n">
-        <v>17</v>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="n">
         <v>0</v>
       </c>
@@ -3300,11 +3244,7 @@
       <c r="E67" t="n">
         <v>7</v>
       </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
         <v>0</v>
       </c>
@@ -3558,11 +3498,7 @@
       <c r="E73" t="n">
         <v>21</v>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" t="n">
         <v>0</v>
       </c>
@@ -3773,11 +3709,7 @@
       <c r="E78" t="n">
         <v>18</v>
       </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="n">
         <v>0</v>
       </c>
@@ -4158,9 +4090,13 @@
         <v>20</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G87" t="n">
         <v>0</v>
       </c>
@@ -4240,9 +4176,13 @@
         <v>14</v>
       </c>
       <c r="E89" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G89" t="n">
         <v>0</v>
       </c>
@@ -4367,11 +4307,7 @@
       <c r="E92" t="n">
         <v>15</v>
       </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
         <v>0</v>
       </c>
@@ -4410,11 +4346,7 @@
       <c r="E93" t="n">
         <v>13</v>
       </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="n">
         <v>0</v>
       </c>
@@ -4453,11 +4385,7 @@
       <c r="E94" t="n">
         <v>12</v>
       </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="n">
         <v>0</v>
       </c>
@@ -4539,11 +4467,7 @@
       <c r="E96" t="n">
         <v>10</v>
       </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="n">
         <v>0</v>
       </c>
@@ -4711,11 +4635,7 @@
       <c r="E100" t="n">
         <v>12</v>
       </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="n">
         <v>0</v>
       </c>
@@ -4881,9 +4801,13 @@
         <v>17</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" t="inlineStr"/>
+        <v>17</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G104" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat: enhance web scraping and error handling in pipeline
- Updated the web scraping process in p1_webscraping.py to extract every second PDF link and merge PDFs from the same main link into a single file.
- Improved error handling and retry logic for PDF merging, ensuring temporary files are cleaned up after processing.
- Enhanced README and MasterSystemPrompt documentation to reflect changes in the web scraping process and error handling strategies.
- Updated performance logs to capture additional metrics related to the new web scraping functionality.
</commit_message>
<xml_diff>
--- a/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
+++ b/inputs/excel/inputExcel/CAO_Frequencies_2014.xlsx
@@ -642,7 +642,11 @@
       <c r="E5" t="n">
         <v>14</v>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
@@ -808,13 +812,9 @@
         <v>13</v>
       </c>
       <c r="E9" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>0</v>
       </c>
@@ -1025,7 +1025,11 @@
       <c r="E14" t="n">
         <v>18</v>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
@@ -1148,13 +1152,9 @@
         <v>16</v>
       </c>
       <c r="E17" t="n">
-        <v>16</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>0</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>36</v>
       </c>
       <c r="E24" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
@@ -1533,7 +1533,11 @@
       <c r="E26" t="n">
         <v>10</v>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
@@ -1615,7 +1619,11 @@
       <c r="E28" t="n">
         <v>26</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
@@ -1654,7 +1662,11 @@
       <c r="E29" t="n">
         <v>13</v>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G29" t="n">
         <v>0</v>
       </c>
@@ -1777,13 +1789,9 @@
         <v>11</v>
       </c>
       <c r="E32" t="n">
-        <v>11</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
         <v>0</v>
       </c>
@@ -1906,7 +1914,7 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
@@ -1990,7 +1998,11 @@
       <c r="E37" t="n">
         <v>4</v>
       </c>
-      <c r="F37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
@@ -2113,7 +2125,7 @@
         <v>20</v>
       </c>
       <c r="E40" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
@@ -2197,7 +2209,11 @@
       <c r="E42" t="n">
         <v>30</v>
       </c>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
@@ -2236,7 +2252,11 @@
       <c r="E43" t="n">
         <v>28</v>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G43" t="n">
         <v>0</v>
       </c>
@@ -2361,7 +2381,11 @@
       <c r="E46" t="n">
         <v>12</v>
       </c>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
@@ -2398,7 +2422,7 @@
         <v>24</v>
       </c>
       <c r="E47" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
@@ -2695,13 +2719,9 @@
         <v>21</v>
       </c>
       <c r="E54" t="n">
-        <v>21</v>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
         <v>0</v>
       </c>
@@ -2996,13 +3016,9 @@
         <v>17</v>
       </c>
       <c r="E61" t="n">
-        <v>17</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="n">
         <v>0</v>
       </c>
@@ -3082,7 +3098,7 @@
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="n">
@@ -3123,7 +3139,11 @@
       <c r="E64" t="n">
         <v>17</v>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G64" t="n">
         <v>0</v>
       </c>
@@ -3205,7 +3225,11 @@
       <c r="E66" t="n">
         <v>0</v>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G66" t="n">
         <v>0</v>
       </c>
@@ -3244,7 +3268,11 @@
       <c r="E67" t="n">
         <v>7</v>
       </c>
-      <c r="F67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G67" t="n">
         <v>0</v>
       </c>
@@ -3283,11 +3311,7 @@
       <c r="E68" t="n">
         <v>0</v>
       </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="n">
         <v>0</v>
       </c>
@@ -3326,11 +3350,7 @@
       <c r="E69" t="n">
         <v>0</v>
       </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="n">
         <v>0</v>
       </c>
@@ -3498,7 +3518,11 @@
       <c r="E73" t="n">
         <v>21</v>
       </c>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G73" t="n">
         <v>0</v>
       </c>
@@ -3709,7 +3733,11 @@
       <c r="E78" t="n">
         <v>18</v>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G78" t="n">
         <v>0</v>
       </c>
@@ -4176,13 +4204,9 @@
         <v>14</v>
       </c>
       <c r="E89" t="n">
-        <v>14</v>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="n">
         <v>0</v>
       </c>
@@ -4307,7 +4331,11 @@
       <c r="E92" t="n">
         <v>15</v>
       </c>
-      <c r="F92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G92" t="n">
         <v>0</v>
       </c>
@@ -4346,7 +4374,11 @@
       <c r="E93" t="n">
         <v>13</v>
       </c>
-      <c r="F93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G93" t="n">
         <v>0</v>
       </c>
@@ -4385,7 +4417,11 @@
       <c r="E94" t="n">
         <v>12</v>
       </c>
-      <c r="F94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G94" t="n">
         <v>0</v>
       </c>
@@ -4422,13 +4458,9 @@
         <v>17</v>
       </c>
       <c r="E95" t="n">
-        <v>17</v>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="n">
         <v>0</v>
       </c>
@@ -4467,7 +4499,11 @@
       <c r="E96" t="n">
         <v>10</v>
       </c>
-      <c r="F96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G96" t="n">
         <v>0</v>
       </c>
@@ -4635,7 +4671,11 @@
       <c r="E100" t="n">
         <v>12</v>
       </c>
-      <c r="F100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G100" t="n">
         <v>0</v>
       </c>
@@ -4715,13 +4755,9 @@
         <v>2</v>
       </c>
       <c r="E102" t="n">
-        <v>2</v>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="n">
         <v>0</v>
       </c>
@@ -4846,11 +4882,7 @@
       <c r="E105" t="n">
         <v>0</v>
       </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="n">
         <v>0</v>
       </c>
@@ -4930,13 +4962,9 @@
         <v>12</v>
       </c>
       <c r="E107" t="n">
-        <v>12</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" t="n">
         <v>0</v>
       </c>
@@ -7606,12 +7634,10 @@
       <c r="D184" t="n">
         <v>5</v>
       </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E184" t="n">
+        <v>5</v>
+      </c>
+      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
@@ -10109,12 +10135,10 @@
       <c r="D257" t="n">
         <v>10</v>
       </c>
-      <c r="E257" t="inlineStr"/>
-      <c r="F257" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E257" t="n">
+        <v>10</v>
+      </c>
+      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr">
         <is>
@@ -11578,12 +11602,10 @@
       <c r="D300" t="n">
         <v>11</v>
       </c>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E300" t="n">
+        <v>11</v>
+      </c>
+      <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr"/>
       <c r="H300" t="inlineStr">
         <is>
@@ -15296,12 +15318,10 @@
       <c r="D408" t="n">
         <v>2</v>
       </c>
-      <c r="E408" t="inlineStr"/>
-      <c r="F408" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E408" t="n">
+        <v>2</v>
+      </c>
+      <c r="F408" t="inlineStr"/>
       <c r="G408" t="inlineStr"/>
       <c r="H408" t="inlineStr">
         <is>
@@ -26204,12 +26224,10 @@
       <c r="D726" t="n">
         <v>12</v>
       </c>
-      <c r="E726" t="inlineStr"/>
-      <c r="F726" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E726" t="n">
+        <v>12</v>
+      </c>
+      <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr"/>
       <c r="H726" t="inlineStr">
         <is>
@@ -26445,12 +26463,10 @@
       <c r="D733" t="n">
         <v>3</v>
       </c>
-      <c r="E733" t="inlineStr"/>
-      <c r="F733" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E733" t="n">
+        <v>3</v>
+      </c>
+      <c r="F733" t="inlineStr"/>
       <c r="G733" t="inlineStr"/>
       <c r="H733" t="inlineStr">
         <is>
@@ -34094,12 +34110,10 @@
       <c r="D956" t="n">
         <v>4</v>
       </c>
-      <c r="E956" t="inlineStr"/>
-      <c r="F956" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E956" t="n">
+        <v>4</v>
+      </c>
+      <c r="F956" t="inlineStr"/>
       <c r="G956" t="inlineStr"/>
       <c r="H956" t="inlineStr">
         <is>
@@ -38317,12 +38331,10 @@
       <c r="D1079" t="n">
         <v>2</v>
       </c>
-      <c r="E1079" t="inlineStr"/>
-      <c r="F1079" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E1079" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1079" t="inlineStr"/>
       <c r="G1079" t="inlineStr"/>
       <c r="H1079" t="inlineStr">
         <is>
@@ -41557,12 +41569,10 @@
       <c r="D1173" t="n">
         <v>3</v>
       </c>
-      <c r="E1173" t="inlineStr"/>
-      <c r="F1173" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E1173" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1173" t="inlineStr"/>
       <c r="G1173" t="inlineStr"/>
       <c r="H1173" t="inlineStr">
         <is>
@@ -55806,12 +55816,10 @@
       <c r="D1588" t="n">
         <v>13</v>
       </c>
-      <c r="E1588" t="inlineStr"/>
-      <c r="F1588" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="E1588" t="n">
+        <v>13</v>
+      </c>
+      <c r="F1588" t="inlineStr"/>
       <c r="G1588" t="inlineStr"/>
       <c r="H1588" t="inlineStr">
         <is>

</xml_diff>